<commit_message>
Continue to update every week
</commit_message>
<xml_diff>
--- a/AI_AuditLog_SWP_NguyenAnhMinh_DE190975.xlsx
+++ b/AI_AuditLog_SWP_NguyenAnhMinh_DE190975.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9060" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12240" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="73">
   <si>
     <t>Entry #</t>
   </si>
@@ -164,6 +164,90 @@
   </si>
   <si>
     <t>Yes (Severe Hallucination &amp; Flawed Logic - AI tự bịa ra điểm số cao cho file trống và CV rác).</t>
+  </si>
+  <si>
+    <t>System Prompt Design &amp; Persona Adoption</t>
+  </si>
+  <si>
+    <t>Implementation (AI Core Engine - CV Scoring System)</t>
+  </si>
+  <si>
+    <t>AI mặc định thường đóng vai trò là một trợ lý thân thiện, dẫn đến việc nhận xét CV chung chung, sáo rỗng và thiếu tính thực chiến. Hệ thống cần một "nhân cách" khó tính, soi lỗi như một nhà tuyển dụng FAANG thực thụ.</t>
+  </si>
+  <si>
+    <t>"You are an elite Senior Technical Recruiter + ATS System + IT Career Mentor with 15+ years of experience... You are STRICT. You DO NOT give fake compliments... Return response in 12 detailed sections (Executive Summary, ATS Analysis, Technical Skills, etc.) with a 100-point scoring system."</t>
+  </si>
+  <si>
+    <t>AI đã nhập vai thành công (Persona adopted), loại bỏ hoàn toàn các câu khen ngợi thừa thãi. Kết quả trả về được định dạng cứng theo đúng 12 mục yêu cầu, chỉ ra trực diện các điểm yếu (Red flags) và tính toán điểm số chính xác theo thang 100 dựa trên 10 tiêu chí đã định nghĩa.</t>
+  </si>
+  <si>
+    <t>Tôi nhận định rằng giá trị cốt lõi của một hệ thống đánh giá CV không nằm ở những lời khen, mà ở việc chỉ ra chính xác điểm chết (Red flags). Tôi chủ động ép AI rũ bỏ sự "dĩ hòa vi quý" để trở nên "tàn nhẫn nhưng thực tế" (brutally honest).</t>
+  </si>
+  <si>
+    <t>Dựa trên thực tế tuyển dụng khốc liệt của ngành IT (FAANG standards, ATS screening), tôi cung cấp bối cảnh rõ ràng để AI hiểu nó đang đóng vai trò gác cổng (Gatekeeper) chứ không phải người tư vấn tâm lý.</t>
+  </si>
+  <si>
+    <t>Các CV ở Việt Nam thường chuộng form của TopCV (2 cột, dùng thanh bar kỹ năng). Tôi đưa 8 mẫu này vào bối cảnh để AI hiểu đặc thù trình bày của ứng viên nội địa, từ đó chấm điểm Layout thực tế hơn.</t>
+  </si>
+  <si>
+    <t>Ứng dụng kỹ thuật Multimodal (Đa phương thức - Kết hợp Text Prompt và Image Input) để thiết lập kỹ thuật Few-Shot Learning. Tôi nạp sẵn dữ liệu đầu vào (Input) đa dạng để "hiệu chỉnh" (Calibrate) lại mức độ khó dễ trong việc cho điểm của AI.</t>
+  </si>
+  <si>
+    <t>Yes (Đã kiểm soát được lỗi Hallucination ảo tưởng sức mạnh, cấm AI tự động sinh ra những lời khen không có căn cứ từ dữ liệu CV).</t>
+  </si>
+  <si>
+    <t>Contextual Constraints &amp; Branching Logic</t>
+  </si>
+  <si>
+    <t>Implementation (AI Core Engine - Ruleset Calibration)</t>
+  </si>
+  <si>
+    <t>Một CV của Frontend Developer không thể được đánh giá bằng cùng một thước đo với CV của DevOps hay AI/ML Engineer. AI cần có bộ luật phân tích (Ruleset) rẽ nhánh riêng biệt cho từng vị trí IT cụ thể.</t>
+  </si>
+  <si>
+    <t>"SPECIAL RULES FOR IT CVs: If role is Frontend focus on React ecosystem, state management, UI/UX... If role is Backend focus on API design, DB design, Scalability, Security... If DevOps evaluate CI/CD, Docker, Kubernetes, Cloud..."</t>
+  </si>
+  <si>
+    <t>AI đã nhận diện được các vị trí ứng tuyển khác nhau và kích hoạt đúng bộ tiêu chí chuyên sâu tương ứng. Ví dụ: Khi phân tích CV Backend, AI tập trung vào đánh giá kiến trúc Caching và API thay vì hỏi về Responsive Design.</t>
+  </si>
+  <si>
+    <t>Tôi phát hiện AI dễ bị đánh lừa bởi việc nhồi nhét từ khóa (Buzzword stuffing) nếu chỉ dùng một bộ lọc IT chung chung. Cần phải có ranh giới rõ ràng giữa các phân hệ (Front/Back/DevOps/AI).</t>
+  </si>
+  <si>
+    <t>Áp dụng kiến thức chuyên ngành Software Engineering thực tế để vạch ra các "điểm chạm" quan trọng nhất của từng vị trí (Ví dụ: DevOps thì phải nói đến Docker/K8s, Frontend thì phải rành State Management).</t>
+  </si>
+  <si>
+    <t>Tích hợp logic rẽ nhánh (If-Else) ngay trong bản thân Prompt. Kỹ thuật này biến một Prompt tĩnh thành một "Functions" linh hoạt, tự điều chỉnh thang đo dựa trên Role khai báo trong CV.</t>
+  </si>
+  <si>
+    <t>Yêu cầu AI phải đánh giá sâu vào kiến trúc (Architecture), bảo mật (Security), và khả năng mở rộng (Scalability) để phân biệt dự án làm theo Tutorial (cấp độ sinh viên) với dự án Production-level (cấp độ đi làm thật).</t>
+  </si>
+  <si>
+    <t>No (AI tuân thủ tuyệt đối các ràng buộc logic rẽ nhánh, không bị lẫn lộn tiêu chí giữa các Role).</t>
+  </si>
+  <si>
+    <t>Few-Shot Prompting &amp; Visual Data Processing</t>
+  </si>
+  <si>
+    <t>Testing &amp; Fine-Tuning (CV Layout &amp; ATS Parsing Performance)</t>
+  </si>
+  <si>
+    <t>AI cần hiểu được các format CV phức tạp phổ biến tại thị trường (đặc biệt là các template hai cột, chứa icon, biểu đồ) để kiểm tra khả năng đọc hiểu của hệ thống quét ATS, đồng thời tạo một "chuẩn đối sánh" (benchmark) về trình độ ứng viên.</t>
+  </si>
+  <si>
+    <t>"And at the same time, based on the following CVs that I will submit here, we can evaluate the criteria more accurately."</t>
+  </si>
+  <si>
+    <t>AI đã phân tích thành công bố cục (Layout) và bóc tách dữ liệu từ 8 bức ảnh CV. AI lưu trữ các mẫu này làm "Base knowledge" (Kiến thức nền) để hiểu rõ sự khác biệt về chất lượng nội dung giữa một CV xịn và một CV kém.</t>
+  </si>
+  <si>
+    <t>Tôi nhận định không thể chỉ Train AI bằng chữ (Text). Để đánh giá tiêu chí "ATS Compatibility" và "Resume Formatting", AI buộc phải được "nhìn" thấy các bản CV thực tế bị lỗi layout, nhồi nhét thông tin hoặc dùng sai font chữ.</t>
+  </si>
+  <si>
+    <t>Quyết định cung cấp hẳn 1 tập dữ liệu (Dataset) nhỏ gồm 8 CV để làm "chuẩn vàng" (Gold standard) thay vì để AI tự đoán mò tiêu chuẩn trình bày.</t>
+  </si>
+  <si>
+    <t>Yes (Lúc đầu AI có thể bị hoa mắt/đọc sai chữ do layout 2 cột phức tạp, nhưng nhờ nạp nhiều ảnh mẫu (Few-shot), AI đã học được cách quét text chính xác theo từng block).</t>
   </si>
 </sst>
 </file>
@@ -193,15 +277,23 @@
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
       <sz val="10"/>
       <color rgb="FF800080"/>
       <name val="Roboto"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
@@ -224,14 +316,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -694,28 +778,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -839,8 +923,32 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -848,18 +956,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -868,12 +970,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -883,7 +979,7 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1292,170 +1388,182 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-        <charset val="134"/>
-        <family val="0"/>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-      </font>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
       <fill>
@@ -1499,7 +1607,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle name="AI_AuditLog_SWP_Template-style" pivot="0" count="4" xr9:uid="{3D066CE8-E913-42A9-9BED-7C92F5D4FDC9}">
+    <tableStyle name="AI_AuditLog_SWP_Template-style" pivot="0" count="4" xr9:uid="{47D42E33-6BA0-4088-B10B-2938AA1E8CDB}">
       <tableStyleElement type="wholeTable" dxfId="38"/>
       <tableStyleElement type="headerRow" dxfId="37"/>
       <tableStyleElement type="firstRowStripe" dxfId="36"/>
@@ -1790,102 +1898,102 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1" spans="1:11">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="16" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" ht="132" customHeight="1" spans="1:11">
-      <c r="A2" s="13">
+      <c r="A2" s="17">
         <v>1</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="K2" s="19" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1" spans="1:11">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
+      <c r="A3" s="20"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:11">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17" t="s">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
     </row>
     <row r="5" ht="22.5" customHeight="1"/>
     <row r="6" ht="22.5" customHeight="1"/>
@@ -1933,136 +2041,136 @@
     <col min="9" max="9" width="46.1111111111111" customWidth="1"/>
     <col min="10" max="10" width="30.5555555555556" customWidth="1"/>
     <col min="11" max="11" width="34.2222222222222" customWidth="1"/>
-    <col min="12" max="12" width="20.6666666666667" style="10" customWidth="1"/>
+    <col min="12" max="12" width="20.6666666666667" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" ht="264" spans="1:12">
-      <c r="A2" s="3">
+    <row r="2" ht="237.6" spans="1:12">
+      <c r="A2" s="4">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="10" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" ht="129" customHeight="1" spans="1:12">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>3</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="K3" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="10" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="2"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="10"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2088,98 +2196,172 @@
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="13.2" outlineLevelRow="3"/>
   <cols>
-    <col min="2" max="2" width="12.2222222222222" customWidth="1"/>
-    <col min="3" max="3" width="16.8888888888889" customWidth="1"/>
-    <col min="4" max="4" width="15.5555555555556" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="23.1111111111111" customWidth="1"/>
-    <col min="7" max="7" width="28.1111111111111" customWidth="1"/>
-    <col min="8" max="8" width="37.2222222222222" customWidth="1"/>
-    <col min="9" max="9" width="26.8888888888889" customWidth="1"/>
-    <col min="10" max="10" width="37.4444444444444" customWidth="1"/>
-    <col min="11" max="11" width="55.3333333333333" customWidth="1"/>
-    <col min="12" max="12" width="84" customWidth="1"/>
+    <col min="1" max="1" width="8.88888888888889" style="1"/>
+    <col min="2" max="2" width="12.2222222222222" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.8888888888889" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5555555555556" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.1111111111111" style="1" customWidth="1"/>
+    <col min="7" max="7" width="28.1111111111111" style="1" customWidth="1"/>
+    <col min="8" max="8" width="37.2222222222222" style="1" customWidth="1"/>
+    <col min="9" max="9" width="26.8888888888889" style="1" customWidth="1"/>
+    <col min="10" max="10" width="37.4444444444444" style="1" customWidth="1"/>
+    <col min="11" max="11" width="55.3333333333333" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.8888888888889" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.88888888888889" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="52.8" spans="1:12">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="26.4" spans="1:12">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="2"/>
+    <row r="2" ht="176" customHeight="1" spans="1:12">
+      <c r="A2" s="4">
+        <v>4</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="3" spans="1:12">
-      <c r="A3" s="6"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="2"/>
+    <row r="3" ht="70" customHeight="1" spans="1:12">
+      <c r="A3" s="3">
+        <v>5</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>64</v>
+      </c>
     </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="2"/>
+    <row r="4" ht="73" customHeight="1" spans="1:12">
+      <c r="A4" s="7">
+        <v>6</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>72</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2187,6 +2369,11 @@
       <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))),AND(ISNUMBER(A2),LEFT(CELL("format",A2))="D")))))</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="K2" r:id="rId2" display="https://docs.google.com/document/d/1eKvFwEUnsxnH7yImOXPAc3Zu7ReY_qVXLsTXpP064lI/edit?tab=t.0"/>
+    <hyperlink ref="K3" r:id="rId2" display="https://docs.google.com/document/d/1eKvFwEUnsxnH7yImOXPAc3Zu7ReY_qVXLsTXpP064lI/edit?tab=t.0"/>
+    <hyperlink ref="K4" r:id="rId2" display="https://docs.google.com/document/d/1eKvFwEUnsxnH7yImOXPAc3Zu7ReY_qVXLsTXpP064lI/edit?tab=t.0"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Update final week : week 9 and week 10
Update final week : week 9 and week 10
</commit_message>
<xml_diff>
--- a/AI_AuditLog_SWP_NguyenAnhMinh_DE190975.xlsx
+++ b/AI_AuditLog_SWP_NguyenAnhMinh_DE190975.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="7"/>
+    <workbookView windowWidth="23040" windowHeight="9000" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="1" r:id="rId1"/>
@@ -15,6 +15,8 @@
     <sheet name="Week 6" sheetId="6" r:id="rId6"/>
     <sheet name="Week 7" sheetId="7" r:id="rId7"/>
     <sheet name="Week 8" sheetId="8" r:id="rId8"/>
+    <sheet name="Week 9" sheetId="9" r:id="rId9"/>
+    <sheet name="Week 10" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="275">
   <si>
     <t>Entry #</t>
   </si>
@@ -793,6 +795,72 @@
   </si>
   <si>
     <t xml:space="preserve"> No (Cấu trúc try-catch fallback cơ bản AI sinh ra là đúng và dễ hiểu).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI/UX Refactoring &amp; Motion Design Integration </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementation (CV Manager - React JSX Overhaul) </t>
+  </si>
+  <si>
+    <t>Giao diện CV Manager ban đầu quá "flat" và tĩnh lặng: khu vực upload chỉ là viền đứt nét, danh sách CV là list cuộn dài mỏi tay. Cần nâng cấp toàn diện layout lên chuẩn SaaS Premium.</t>
+  </si>
+  <si>
+    <t>Tôi muốn tích hợp thư viện Aceternity UI (Bento Grid, Kinetic Upload) và Framer Motion vào CVManager. Hãy cấu trúc lại phần JSX mà KHÔNG ảnh hưởng đến logic AI phía trên."</t>
+  </si>
+  <si>
+    <t>AI lên kế hoạch: Cài `framer-motion`, `lucide-react`; tái cấu trúc phần JSX cuối file thành Kinetic Upload Portal với Spring Animations (`whileHover`, `whileTap`).</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Yêu cầu giữ nguyên 100% hệ màu "Clean Tech" (Kem, Trắng, Xám, Vàng Cát) — bác bỏ đề xuất Dark Mode/Neon mặc định của Aceternity UI. </t>
+  </si>
+  <si>
+    <t>Áp dụng Spring Animations (`type: 'spring', stiffness: 400, damping: 25`) cho Drop Zone. Tái cấu trúc grid hiển thị Bento UI.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tự tích hợp Aceternity-style grid background pattern (24px) bằng thẻ SVG inline. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiên quyết chỉ "phẫu thuật" phần vỏ bọc JSX (return statement), giữ nguyên 100% logic AI/Supabase ở phần trên. Xác nhận không ảnh hưởng API integrations. </t>
+  </si>
+  <si>
+    <t>`CVManager.jsx`, `package.json`</t>
+  </si>
+  <si>
+    <t>No (AI tách đúng phần UI ra khỏi logic AI).</t>
+  </si>
+  <si>
+    <t>Advanced Data Visualization &amp; CSS Styling</t>
+  </si>
+  <si>
+    <t>Implementation (CV Manager - CSS &amp; Graphic Elements)</t>
+  </si>
+  <si>
+    <t>File CSS cũ không còn phù hợp với cấu trúc Bento Grid. Cần viết lại toàn bộ CSS, bổ sung các component đồ họa SVG nâng cao (Sparkle Button, ATS Score Ring).</t>
+  </si>
+  <si>
+    <t>"Hãy viết file CSS hoàn chỉnh cho giao diện Bento Grid mới dựa trên hệ màu Clean Tech. Thêm nút Sparkle Button với hiệu ứng particle và vòng tròn ATS Score."</t>
+  </si>
+  <si>
+    <t>AI sinh toàn bộ CSS class tương ứng và code inline SVG cho Sparkle Button (Uiverse) và ATS Ring</t>
+  </si>
+  <si>
+    <t>AI viết code CSS quá dài và đôi chỗ lặp class. Tôi tự cấu trúc lại CSS thành các block BEM rõ ràng để dễ bảo trì.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Định nghĩa lại các thẻ CSS Variables (`--color-cream`, `--color-accent`) ở đầu file để đồng bộ màu sắc toàn trang. </t>
+  </si>
+  <si>
+    <t>Tích hợp Sparkle Button (10 particle effects bằng SVG inline) và ATS Score Ring hiển thị gradient 3 màu siêu mượt.</t>
+  </si>
+  <si>
+    <t>Tự thiết kế các hiệu ứng CSS Shimmer loading cho phần chờ AI phân tích thay vì dùng ảnh GIF để tối ưu hiệu suất.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> `CVManager.css` (2156 dòng)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> No (AI sinh mã CSS và SVG chuẩn xác).</t>
   </si>
 </sst>
 </file>
@@ -1594,7 +1662,7 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="99">
+  <dxfs count="123">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -2793,6 +2861,342 @@
       <font>
         <name val="Arial"/>
         <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="none"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+        <charset val="134"/>
+        <family val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <scheme val="minor"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -3013,11 +3417,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle name="AI_AuditLog_SWP_Template-style" pivot="0" count="4" xr9:uid="{66674EFA-5461-4A16-9642-2C65AE51425D}">
-      <tableStyleElement type="wholeTable" dxfId="98"/>
-      <tableStyleElement type="headerRow" dxfId="97"/>
-      <tableStyleElement type="firstRowStripe" dxfId="96"/>
-      <tableStyleElement type="secondRowStripe" dxfId="95"/>
+    <tableStyle name="AI_AuditLog_SWP_Template-style" pivot="0" count="4" xr9:uid="{36CB1639-94EB-4D64-ADF1-764A90D30A41}">
+      <tableStyleElement type="wholeTable" dxfId="122"/>
+      <tableStyleElement type="headerRow" dxfId="121"/>
+      <tableStyleElement type="firstRowStripe" dxfId="120"/>
+      <tableStyleElement type="secondRowStripe" dxfId="119"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -3042,6 +3446,26 @@
     <tableColumn id="9" name="Human Delta: Creative Synthesis" dataDxfId="8"/>
     <tableColumn id="10" name="Human Delta: Decision Ownership" dataDxfId="9"/>
     <tableColumn id="11" name="Evidence" dataDxfId="10"/>
+  </tableColumns>
+  <tableStyleInfo name="AI_AuditLog_SWP_Template-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="SWP_345678911" displayName="SWP_345678911" ref="A1:L4">
+  <tableColumns count="12">
+    <tableColumn id="1" name="Entry #" dataDxfId="107"/>
+    <tableColumn id="2" name="Prompt Type" dataDxfId="108"/>
+    <tableColumn id="3" name="Stage/Component" dataDxfId="109"/>
+    <tableColumn id="4" name="Problem/Context" dataDxfId="110"/>
+    <tableColumn id="5" name="Prompt to AI" dataDxfId="111"/>
+    <tableColumn id="6" name="AI Response (Summary)" dataDxfId="112"/>
+    <tableColumn id="7" name="Human Delta: Critical Thinking" dataDxfId="113"/>
+    <tableColumn id="8" name="Human Delta: Contextualization" dataDxfId="114"/>
+    <tableColumn id="9" name="Human Delta: Creative Synthesis" dataDxfId="115"/>
+    <tableColumn id="10" name="Human Delta: Decision Ownership" dataDxfId="116"/>
+    <tableColumn id="11" name="Evidence" dataDxfId="117"/>
+    <tableColumn id="12" name="Hallucination Detected?" dataDxfId="118"/>
   </tableColumns>
   <tableStyleInfo name="AI_AuditLog_SWP_Template-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3182,6 +3606,26 @@
     <tableColumn id="10" name="Human Delta: Decision Ownership" dataDxfId="92"/>
     <tableColumn id="11" name="Evidence" dataDxfId="93"/>
     <tableColumn id="12" name="Hallucination Detected?" dataDxfId="94"/>
+  </tableColumns>
+  <tableStyleInfo name="AI_AuditLog_SWP_Template-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="SWP_345678910" displayName="SWP_345678910" ref="A1:L2">
+  <tableColumns count="12">
+    <tableColumn id="1" name="Entry #" dataDxfId="95"/>
+    <tableColumn id="2" name="Prompt Type" dataDxfId="96"/>
+    <tableColumn id="3" name="Stage/Component" dataDxfId="97"/>
+    <tableColumn id="4" name="Problem/Context" dataDxfId="98"/>
+    <tableColumn id="5" name="Prompt to AI" dataDxfId="99"/>
+    <tableColumn id="6" name="AI Response (Summary)" dataDxfId="100"/>
+    <tableColumn id="7" name="Human Delta: Critical Thinking" dataDxfId="101"/>
+    <tableColumn id="8" name="Human Delta: Contextualization" dataDxfId="102"/>
+    <tableColumn id="9" name="Human Delta: Creative Synthesis" dataDxfId="103"/>
+    <tableColumn id="10" name="Human Delta: Decision Ownership" dataDxfId="104"/>
+    <tableColumn id="11" name="Evidence" dataDxfId="105"/>
+    <tableColumn id="12" name="Hallucination Detected?" dataDxfId="106"/>
   </tableColumns>
   <tableStyleInfo name="AI_AuditLog_SWP_Template-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3530,6 +3974,147 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="13.2" outlineLevelRow="3"/>
+  <cols>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="20.8888888888889" customWidth="1"/>
+    <col min="4" max="4" width="41.2222222222222" customWidth="1"/>
+    <col min="5" max="5" width="58.6666666666667" customWidth="1"/>
+    <col min="6" max="6" width="42" customWidth="1"/>
+    <col min="7" max="7" width="40.7777777777778" customWidth="1"/>
+    <col min="8" max="8" width="29.6666666666667" customWidth="1"/>
+    <col min="9" max="9" width="35.7777777777778" customWidth="1"/>
+    <col min="10" max="10" width="32.8888888888889" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="26.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" s="3"/>
+    </row>
+    <row r="2" ht="120" customHeight="1" spans="1:13">
+      <c r="A2" s="4">
+        <v>26</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" ht="13.8" spans="1:13">
+      <c r="A3" s="4"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" ht="88" customHeight="1" spans="1:13">
+      <c r="A4" s="4"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="3"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="custom" allowBlank="1" sqref="A2:A4">
+      <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))),AND(ISNUMBER(A2),LEFT(CELL("format",A2))="D")))))</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
@@ -4794,7 +5379,7 @@
     <col min="12" max="12" width="26.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26.4" spans="1:13">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4967,4 +5552,124 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="13.2" outlineLevelRow="3"/>
+  <cols>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="20.8888888888889" customWidth="1"/>
+    <col min="4" max="4" width="41.2222222222222" customWidth="1"/>
+    <col min="5" max="5" width="58.6666666666667" customWidth="1"/>
+    <col min="6" max="6" width="42" customWidth="1"/>
+    <col min="7" max="7" width="40.7777777777778" customWidth="1"/>
+    <col min="8" max="8" width="29.6666666666667" customWidth="1"/>
+    <col min="9" max="9" width="35.7777777777778" customWidth="1"/>
+    <col min="10" max="10" width="32.8888888888889" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="26.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" s="3"/>
+    </row>
+    <row r="2" ht="120" customHeight="1" spans="1:13">
+      <c r="A2" s="4">
+        <v>25</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" ht="104" customHeight="1" spans="1:13">
+      <c r="M4" s="3"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="custom" allowBlank="1" sqref="A2">
+      <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))),AND(ISNUMBER(A2),LEFT(CELL("format",A2))="D")))))</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="K2" r:id="rId2" display="`CVManager.jsx`, `package.json`" tooltip="https://docs.google.com/document/d/1eKvFwEUnsxnH7yImOXPAc3Zu7ReY_qVXLsTXpP064lI/edit?tab=t.0"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>